<commit_message>
Update daily BIST tracking Excel
</commit_message>
<xml_diff>
--- a/Yüzde .xlsx
+++ b/Yüzde .xlsx
@@ -6,8 +6,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="VERİLER" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="BIST" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ÖZET" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="VERİLER" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BIST" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -813,6 +814,154 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Alan</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Değer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Son Güncelleme</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>30.06.2026 10:21:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Veri Kaynağı</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>tradingview</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Fallback</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>KAPALI</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Yeni AL</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Güncellenen Satır</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Yeni Kapanan İşlem</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Toplam İşlem</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Açık İşlem</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>STOP İşlem</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>KAR STOP İşlem</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Script Versiyon</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>tarama.py 2026-06-08 ESv4-revised</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Y26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
@@ -1006,7 +1155,7 @@
         </is>
       </c>
       <c r="L2" s="8" t="n">
-        <v>23.54</v>
+        <v>23.74</v>
       </c>
       <c r="M2" s="8" t="n">
         <v>-4.62</v>
@@ -1040,7 +1189,7 @@
         <v>-4.61</v>
       </c>
       <c r="X2" s="8" t="n">
-        <v>-14.9</v>
+        <v>-14.17</v>
       </c>
       <c r="Y2" s="9" t="n"/>
     </row>
@@ -1168,7 +1317,7 @@
         </is>
       </c>
       <c r="L4" s="8" t="n">
-        <v>183</v>
+        <v>183.4</v>
       </c>
       <c r="M4" s="8" t="n">
         <v>-4.98</v>
@@ -1202,7 +1351,7 @@
         <v>-10.76</v>
       </c>
       <c r="X4" s="8" t="n">
-        <v>-4.14</v>
+        <v>-3.93</v>
       </c>
       <c r="Y4" s="9" t="n"/>
     </row>
@@ -1249,7 +1398,7 @@
         </is>
       </c>
       <c r="L5" s="5" t="n">
-        <v>13.47</v>
+        <v>13.24</v>
       </c>
       <c r="M5" s="5" t="n">
         <v>8.470000000000001</v>
@@ -1328,7 +1477,7 @@
         </is>
       </c>
       <c r="L6" s="8" t="n">
-        <v>7.2</v>
+        <v>6.95</v>
       </c>
       <c r="M6" s="8" t="n">
         <v>27.27</v>
@@ -1407,7 +1556,7 @@
         </is>
       </c>
       <c r="L7" s="5" t="n">
-        <v>70.5</v>
+        <v>72.95</v>
       </c>
       <c r="M7" s="5" t="n">
         <v>-4.98</v>
@@ -1441,7 +1590,7 @@
         <v>-10.43</v>
       </c>
       <c r="X7" s="5" t="n">
-        <v>-9.85</v>
+        <v>-6.71</v>
       </c>
       <c r="Y7" s="6" t="n"/>
     </row>
@@ -1488,7 +1637,7 @@
         </is>
       </c>
       <c r="L8" s="8" t="n">
-        <v>24.1</v>
+        <v>23.92</v>
       </c>
       <c r="M8" s="8" t="n">
         <v>-4.99</v>
@@ -1501,13 +1650,13 @@
         <v>28.92</v>
       </c>
       <c r="Q8" s="8" t="n">
-        <v>24.06</v>
+        <v>23.88</v>
       </c>
       <c r="R8" s="8" t="n">
         <v>7.67</v>
       </c>
       <c r="S8" s="8" t="n">
-        <v>-10.42</v>
+        <v>-11.09</v>
       </c>
       <c r="T8" s="8" t="n">
         <v>13938.48</v>
@@ -1522,7 +1671,7 @@
         <v>-8.449999999999999</v>
       </c>
       <c r="X8" s="8" t="n">
-        <v>-5.56</v>
+        <v>-6.27</v>
       </c>
       <c r="Y8" s="9" t="n"/>
     </row>
@@ -1569,7 +1718,7 @@
         </is>
       </c>
       <c r="L9" s="5" t="n">
-        <v>43.22</v>
+        <v>43.14</v>
       </c>
       <c r="M9" s="5" t="n">
         <v>-5.01</v>
@@ -1603,7 +1752,7 @@
         <v>-5.66</v>
       </c>
       <c r="X9" s="5" t="n">
-        <v>-6.65</v>
+        <v>-6.83</v>
       </c>
       <c r="Y9" s="6" t="n"/>
     </row>
@@ -1650,7 +1799,7 @@
         </is>
       </c>
       <c r="L10" s="8" t="n">
-        <v>40.26</v>
+        <v>40.58</v>
       </c>
       <c r="M10" s="8" t="n">
         <v>-5.01</v>
@@ -1684,7 +1833,7 @@
         <v>-4.51</v>
       </c>
       <c r="X10" s="8" t="n">
-        <v>-8.5</v>
+        <v>-7.77</v>
       </c>
       <c r="Y10" s="9" t="n"/>
     </row>
@@ -1812,7 +1961,7 @@
         </is>
       </c>
       <c r="L12" s="8" t="n">
-        <v>115</v>
+        <v>115.2</v>
       </c>
       <c r="M12" s="8" t="n">
         <v>-5.02</v>
@@ -1825,13 +1974,13 @@
         <v>134.1</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="R12" s="8" t="n">
         <v>5.26</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>-9.73</v>
+        <v>-10.52</v>
       </c>
       <c r="T12" s="8" t="n">
         <v>14493.09</v>
@@ -1846,7 +1995,7 @@
         <v>-4.52</v>
       </c>
       <c r="X12" s="8" t="n">
-        <v>-4.96</v>
+        <v>-4.79</v>
       </c>
       <c r="Y12" s="9" t="n"/>
     </row>
@@ -1893,7 +2042,7 @@
         </is>
       </c>
       <c r="L13" s="5" t="n">
-        <v>150.7</v>
+        <v>151</v>
       </c>
       <c r="M13" s="5" t="n">
         <v>-4.98</v>
@@ -1903,13 +2052,13 @@
         <v>1</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>150.7</v>
+        <v>155</v>
       </c>
       <c r="Q13" s="5" t="n">
         <v>118.5</v>
       </c>
       <c r="R13" s="5" t="n">
-        <v>17.28</v>
+        <v>20.62</v>
       </c>
       <c r="S13" s="5" t="n">
         <v>-7.78</v>
@@ -1927,7 +2076,7 @@
         <v>-7.8</v>
       </c>
       <c r="X13" s="5" t="n">
-        <v>23.42</v>
+        <v>23.67</v>
       </c>
       <c r="Y13" s="6" t="n"/>
     </row>
@@ -1974,7 +2123,7 @@
         </is>
       </c>
       <c r="L14" s="8" t="n">
-        <v>20.08</v>
+        <v>19.73</v>
       </c>
       <c r="M14" s="8" t="n">
         <v>-5.01</v>
@@ -2008,7 +2157,7 @@
         <v>-3.69</v>
       </c>
       <c r="X14" s="8" t="n">
-        <v>15.07</v>
+        <v>13.07</v>
       </c>
       <c r="Y14" s="9" t="n"/>
     </row>
@@ -2055,7 +2204,7 @@
         </is>
       </c>
       <c r="L15" s="5" t="n">
-        <v>70.55</v>
+        <v>68.34999999999999</v>
       </c>
       <c r="M15" s="5" t="n">
         <v>-5.01</v>
@@ -2089,7 +2238,7 @@
         <v>-4.98</v>
       </c>
       <c r="X15" s="5" t="n">
-        <v>9.460000000000001</v>
+        <v>6.05</v>
       </c>
       <c r="Y15" s="6" t="n"/>
     </row>
@@ -2128,14 +2277,14 @@
       <c r="J16" s="8" t="n"/>
       <c r="K16" s="9" t="n"/>
       <c r="L16" s="8" t="n">
-        <v>136.8</v>
+        <v>138.9</v>
       </c>
       <c r="M16" s="8" t="n"/>
       <c r="N16" s="8" t="n">
-        <v>10.32</v>
+        <v>12.02</v>
       </c>
       <c r="O16" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P16" s="8" t="n">
         <v>140.9</v>
@@ -2159,7 +2308,7 @@
         <v>-3.09</v>
       </c>
       <c r="W16" s="8" t="n">
-        <v>13.41</v>
+        <v>15.11</v>
       </c>
       <c r="X16" s="8" t="n"/>
       <c r="Y16" s="9" t="n"/>
@@ -2207,7 +2356,7 @@
         </is>
       </c>
       <c r="L17" s="5" t="n">
-        <v>85.09999999999999</v>
+        <v>85</v>
       </c>
       <c r="M17" s="5" t="n">
         <v>-5.02</v>
@@ -2241,7 +2390,7 @@
         <v>-3.59</v>
       </c>
       <c r="X17" s="5" t="n">
-        <v>-11.81</v>
+        <v>-11.92</v>
       </c>
       <c r="Y17" s="6" t="n"/>
     </row>
@@ -2288,7 +2437,7 @@
         </is>
       </c>
       <c r="L18" s="8" t="n">
-        <v>4.61</v>
+        <v>4.64</v>
       </c>
       <c r="M18" s="8" t="n">
         <v>-4.91</v>
@@ -2322,7 +2471,7 @@
         <v>-3.48</v>
       </c>
       <c r="X18" s="8" t="n">
-        <v>-4.75</v>
+        <v>-4.13</v>
       </c>
       <c r="Y18" s="9" t="n"/>
     </row>
@@ -2361,14 +2510,14 @@
       <c r="J19" s="5" t="n"/>
       <c r="K19" s="6" t="n"/>
       <c r="L19" s="5" t="n">
-        <v>19.25</v>
+        <v>19.37</v>
       </c>
       <c r="M19" s="5" t="n"/>
       <c r="N19" s="5" t="n">
-        <v>-2.68</v>
+        <v>-2.07</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P19" s="5" t="n">
         <v>20.44</v>
@@ -2392,7 +2541,7 @@
         <v>-0.4</v>
       </c>
       <c r="W19" s="5" t="n">
-        <v>-2.28</v>
+        <v>-1.67</v>
       </c>
       <c r="X19" s="5" t="n"/>
       <c r="Y19" s="6" t="n"/>
@@ -2440,7 +2589,7 @@
         </is>
       </c>
       <c r="L20" s="8" t="n">
-        <v>7.34</v>
+        <v>7.27</v>
       </c>
       <c r="M20" s="8" t="n">
         <v>-5</v>
@@ -2474,7 +2623,7 @@
         <v>-5.1</v>
       </c>
       <c r="X20" s="8" t="n">
-        <v>4.41</v>
+        <v>3.41</v>
       </c>
       <c r="Y20" s="9" t="n"/>
     </row>
@@ -2513,14 +2662,14 @@
       <c r="J21" s="5" t="n"/>
       <c r="K21" s="6" t="n"/>
       <c r="L21" s="5" t="n">
-        <v>5.33</v>
+        <v>5.18</v>
       </c>
       <c r="M21" s="5" t="n"/>
       <c r="N21" s="5" t="n">
-        <v>3.5</v>
+        <v>0.58</v>
       </c>
       <c r="O21" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P21" s="5" t="n">
         <v>5.5</v>
@@ -2544,7 +2693,7 @@
         <v>0.1</v>
       </c>
       <c r="W21" s="5" t="n">
-        <v>3.4</v>
+        <v>0.48</v>
       </c>
       <c r="X21" s="5" t="n"/>
       <c r="Y21" s="6" t="n"/>
@@ -2592,7 +2741,7 @@
         </is>
       </c>
       <c r="L22" s="8" t="n">
-        <v>1.91</v>
+        <v>1.92</v>
       </c>
       <c r="M22" s="8" t="n">
         <v>-3.41</v>
@@ -2626,7 +2775,7 @@
         <v>-3.51</v>
       </c>
       <c r="X22" s="8" t="n">
-        <v>-3.54</v>
+        <v>-3.03</v>
       </c>
       <c r="Y22" s="9" t="n"/>
     </row>
@@ -2665,26 +2814,26 @@
       <c r="J23" s="5" t="n"/>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="5" t="n">
-        <v>29.38</v>
+        <v>29.08</v>
       </c>
       <c r="M23" s="5" t="n"/>
       <c r="N23" s="5" t="n">
-        <v>-2.07</v>
+        <v>-3.07</v>
       </c>
       <c r="O23" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P23" s="5" t="n">
         <v>30.2</v>
       </c>
       <c r="Q23" s="5" t="n">
-        <v>29.24</v>
+        <v>29.08</v>
       </c>
       <c r="R23" s="5" t="n">
         <v>0.67</v>
       </c>
       <c r="S23" s="5" t="n">
-        <v>-2.53</v>
+        <v>-3.07</v>
       </c>
       <c r="T23" s="5" t="n">
         <v>14274.02</v>
@@ -2696,7 +2845,7 @@
         <v>0</v>
       </c>
       <c r="W23" s="5" t="n">
-        <v>-2.07</v>
+        <v>-3.07</v>
       </c>
       <c r="X23" s="5" t="n"/>
       <c r="Y23" s="6" t="n"/>
@@ -2732,25 +2881,25 @@
         </is>
       </c>
       <c r="L24" t="n">
-        <v>5365</v>
+        <v>5425</v>
       </c>
       <c r="N24" t="n">
-        <v>0</v>
+        <v>1.12</v>
       </c>
       <c r="O24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P24" t="n">
-        <v>5680</v>
+        <v>5425</v>
       </c>
       <c r="Q24" t="n">
-        <v>5260</v>
+        <v>5310</v>
       </c>
       <c r="R24" t="n">
-        <v>5.87</v>
+        <v>1.12</v>
       </c>
       <c r="S24" t="n">
-        <v>-1.96</v>
+        <v>-1.03</v>
       </c>
       <c r="T24" t="n">
         <v>14274.02</v>
@@ -2762,7 +2911,7 @@
         <v>0</v>
       </c>
       <c r="W24" t="n">
-        <v>0</v>
+        <v>1.12</v>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
@@ -2801,25 +2950,25 @@
         </is>
       </c>
       <c r="L25" t="n">
-        <v>20.16</v>
+        <v>20</v>
       </c>
       <c r="N25" t="n">
-        <v>0</v>
+        <v>-0.79</v>
       </c>
       <c r="O25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P25" t="n">
-        <v>21.6</v>
+        <v>20.6</v>
       </c>
       <c r="Q25" t="n">
-        <v>19.62</v>
+        <v>19.96</v>
       </c>
       <c r="R25" t="n">
-        <v>7.14</v>
+        <v>2.18</v>
       </c>
       <c r="S25" t="n">
-        <v>-2.68</v>
+        <v>-0.99</v>
       </c>
       <c r="T25" t="n">
         <v>14274.02</v>
@@ -2831,7 +2980,7 @@
         <v>0</v>
       </c>
       <c r="W25" t="n">
-        <v>0</v>
+        <v>-0.79</v>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
@@ -2870,25 +3019,25 @@
         </is>
       </c>
       <c r="L26" t="n">
-        <v>99.05</v>
+        <v>99.5</v>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="O26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P26" t="n">
-        <v>99.40000000000001</v>
+        <v>99.55</v>
       </c>
       <c r="Q26" t="n">
-        <v>97.45</v>
+        <v>99</v>
       </c>
       <c r="R26" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="S26" t="n">
-        <v>-1.62</v>
+        <v>-0.05</v>
       </c>
       <c r="T26" t="n">
         <v>14274.02</v>
@@ -2900,7 +3049,7 @@
         <v>0</v>
       </c>
       <c r="W26" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
@@ -2917,7 +3066,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>